<commit_message>
Updated test bundle gen
</commit_message>
<xml_diff>
--- a/tests/data/scaffolding/v2/phenotype_HIVIND20_filled.xlsx
+++ b/tests/data/scaffolding/v2/phenotype_HIVIND20_filled.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pmanko/code/who_l3_smart_tools/tests/data/scaffolding/v2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{213B5256-C1CD-F048-A3C3-D28740BA3542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3950892-369B-244C-9C5F-7D1882E51C02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="880" windowWidth="41120" windowHeight="23780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="41120" windowHeight="19660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>